<commit_message>
Add a plant-wise grid under the make list, same tab
Plants down the side, tube thickness across the top, MT in the cell, then
TOTAL / W1 / W2. A pure aggregation of the 44 lines above it -- nothing
added, and it ties out both ways: rows and columns each sum to 509.21,
and W1 426.14 + W2 83.07 matches the rolling plan's slots (South W1
179.14, West W1 247.00, West W2 83.07).

A blank cell means that plant makes nothing at that thickness this cycle,
which is most of the grid: NPMD carries 1.6, 2.5 and 3 mm only, Tapi 3, 4
and 5 mm, and the two South plants between them cover 1.6 to 4 mm.

The previous PASS stamp is stale by construction -- the file changed, so
the hash no longer matches. Re-verification is in flight and the file is
not sent until it clears.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFHPZZgkCQmV9B7a9QKcP2
</commit_message>
<xml_diff>
--- a/reports/Make-List-NoStock-2026-10-26.xlsx
+++ b/reports/Make-List-NoStock-2026-10-26.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -94,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,6 +116,12 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -477,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2030,6 +2040,241 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>THE PLAN, PLANT BY PLANT — MT of tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Same 509.21 MT, nothing added. Columns are the tube thickness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t>Plant</t>
+        </is>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>1.6 mm</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>2 mm</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>2.5 mm</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>2.8 mm</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>3 mm</t>
+        </is>
+      </c>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>4 mm</t>
+        </is>
+      </c>
+      <c r="H58" s="16" t="inlineStr">
+        <is>
+          <t>5 mm</t>
+        </is>
+      </c>
+      <c r="I58" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="J58" s="16" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="K58" s="16" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="C59" s="11" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="D59" s="11" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="E59" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F59" s="11" t="n">
+        <v>23.15</v>
+      </c>
+      <c r="G59" s="11" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="H59" s="11" t="n"/>
+      <c r="I59" s="18" t="n">
+        <v>119.35</v>
+      </c>
+      <c r="J59" s="11" t="n">
+        <v>119.35</v>
+      </c>
+      <c r="K59" s="11" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Lepakshi</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="n"/>
+      <c r="C60" s="11" t="n">
+        <v>26.13</v>
+      </c>
+      <c r="D60" s="11" t="n">
+        <v>18.53</v>
+      </c>
+      <c r="E60" s="11" t="n"/>
+      <c r="F60" s="11" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="G60" s="11" t="n">
+        <v>8.27</v>
+      </c>
+      <c r="H60" s="11" t="n"/>
+      <c r="I60" s="18" t="n">
+        <v>59.79</v>
+      </c>
+      <c r="J60" s="11" t="n">
+        <v>59.79</v>
+      </c>
+      <c r="K60" s="11" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>NPMD</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="C61" s="11" t="n"/>
+      <c r="D61" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="E61" s="11" t="n"/>
+      <c r="F61" s="11" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="G61" s="11" t="n"/>
+      <c r="H61" s="11" t="n"/>
+      <c r="I61" s="18" t="n">
+        <v>256.1</v>
+      </c>
+      <c r="J61" s="11" t="n">
+        <v>202.1</v>
+      </c>
+      <c r="K61" s="11" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>Tapi</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="n"/>
+      <c r="C62" s="11" t="n"/>
+      <c r="D62" s="11" t="n"/>
+      <c r="E62" s="11" t="n"/>
+      <c r="F62" s="11" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G62" s="11" t="n">
+        <v>59.07</v>
+      </c>
+      <c r="H62" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="I62" s="18" t="n">
+        <v>73.97</v>
+      </c>
+      <c r="J62" s="11" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="K62" s="11" t="n">
+        <v>29.07</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="n">
+        <v>160.14</v>
+      </c>
+      <c r="C63" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D63" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="E63" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="F63" s="18" t="n">
+        <v>113</v>
+      </c>
+      <c r="G63" s="18" t="n">
+        <v>81.06999999999999</v>
+      </c>
+      <c r="H63" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="I63" s="18" t="n">
+        <v>509.21</v>
+      </c>
+      <c r="J63" s="18" t="n">
+        <v>426.14</v>
+      </c>
+      <c r="K63" s="18" t="n">
+        <v>83.06999999999999</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Blank cell = that plant makes nothing at that thickness this cycle. South is Hyderabad + Lepakshi, West is NPMD + Tapi; a plant only ever makes for its own region.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:G48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>